<commit_message>
comparativo: aba CMD x br-core-composition e origem das restrições
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UVSEtwhqSH6xEBzE8dBMwP
</commit_message>
<xml_diff>
--- a/comparativo/comparativo_sumarioalta_rnds_brcore.xlsx
+++ b/comparativo/comparativo_sumarioalta_rnds_brcore.xlsx
@@ -8,14 +8,16 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composition" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seções" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Débitos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CMD × br-core-composition" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composition" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seções" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Débitos" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Composition'!$A$1:$P$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seções'!$A$1:$P$125</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Débitos'!$A$1:$E$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CMD × br-core-composition'!$A$1:$K$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Composition'!$A$1:$R$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Seções'!$A$1:$R$125</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Débitos'!$A$1:$E$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -518,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -537,90 +539,90 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Herança</t>
+          <t>Cadeias de herança comparadas</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>SA-IG: BRSumarioAlta → BRConjuntoMinimoDados-1.1 (CMD) → Composition (R4). Canonical http://www.saude.gov.br/fhir/r4, sem dependência do BR-Core.</t>
+          <t>Nível 1, documento-base: BRConjuntoMinimoDados-1.1 (CMD) × br-core-composition. Aba "CMD × br-core-composition".</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BR-Core: br-core-sumarioalta → br-core-composition → Composition (R4). Canonical https://br-core.saude.gov.br/fhir.</t>
+          <t>Nível 2, Sumário de Alta: BRSumarioAlta × br-core-sumarioalta. Abas "Composition" e "Seções"; as colunas "Origem da restrição" dizem em que nível cada regra foi declarada.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Sumário de Alta refatorado (IG InspiraSA): usa o br-core-sumarioalta sem perfil próprio. Cadeia: br-core-sumarioalta → br-core-composition → Composition (R4), a mesma do BR-Core. O CMD sai da cadeia.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Fontes</t>
-        </is>
-      </c>
+      <c r="A7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>SA-IG: StructureDefinition-BRSumarioAlta.json (snapshot) do repositório sa-ig.</t>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Herança</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>BR-Core 1.3.0: pacote br.gov.saude.br-core.fhir#1.3.0 (snapshot).</t>
+          <t>SA-IG: BRSumarioAlta → BRConjuntoMinimoDados-1.1 (CMD) → Composition (R4). Canonical http://www.saude.gov.br/fhir/r4, sem dependência do BR-Core.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BR-Core corrigido: branch fix/sumarioalta-capacidadefuncional do repositório br.org.hl7.fhir.core (snapshot gerado pelo SUSHI 3.20.1), ainda não publicado.</t>
+          <t>BR-Core: br-core-sumarioalta → br-core-composition → Composition (R4). Canonical https://br-core.saude.gov.br/fhir.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>FHIR R4: hl7.fhir.r4.core#4.0.1.</t>
-        </is>
-      </c>
+      <c r="A11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Fontes</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Abas</t>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>SA-IG: StructureDefinition-BRSumarioAlta.json (snapshot) do repositório sa-ig.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Composition: elementos do cabeçalho do documento.</t>
+          <t>BR-Core 1.3.0: pacote br.gov.saude.br-core.fhir#1.3.0 (snapshot).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Seções: correspondência entre as 9 seções do SA-IG e as 7 do BR-Core, com os subelementos de cada seção.</t>
+          <t>BR-Core corrigido: branch fix/sumarioalta-capacidadefuncional do repositório br.org.hl7.fhir.core (snapshot gerado pelo SUSHI 3.20.1), ainda não publicado.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Débitos: lista consolidada, por grau.</t>
+          <t>FHIR R4: hl7.fhir.r4.core#4.0.1.</t>
         </is>
       </c>
     </row>
@@ -630,39 +632,70 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Conformidade (documento SA-IG validado contra o br-core-sumarioalta)</t>
+          <t>Abas</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Não conforme: o SA-IG proíbe o que o BR-Core exige, permite omitir o que o BR-Core exige, permite mais ocorrências do que o BR-Core aceita, ou usa outro ValueSet onde o BR-Core é required. Divergente: restrições diferentes que não impedem, por si, a validação. Conforme: mesma cardinalidade e mesmas restrições. Sem equivalente: o elemento existe só em um dos modelos.</t>
+          <t>Composition: elementos do cabeçalho do documento.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Seções: correspondência entre as 9 seções do SA-IG e as 7 do BR-Core, com os subelementos de cada seção.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Grau</t>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Débitos: lista consolidada, por grau.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Bloqueante: impede instância válida. Alto: quebra conformidade ou interoperabilidade. Médio: ambiguidade. Baixo: ajuste de documentação.</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Conformidade (documento SA-IG validado contra o br-core-sumarioalta)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Não conforme: o SA-IG proíbe o que o BR-Core exige, permite omitir o que o BR-Core exige, permite mais ocorrências do que o BR-Core aceita, ou usa outro ValueSet onde o BR-Core é required. Divergente: restrições diferentes que não impedem, por si, a validação. Conforme: mesma cardinalidade e mesmas restrições. Sem equivalente: o elemento existe só em um dos modelos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Grau</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Bloqueante: impede instância válida. Alto: quebra conformidade ou interoperabilidade. Médio: ambiguidade. Baixo: ajuste de documentação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Gerado em 06/10/2026. Autoria: Jussara Macedo Pinho Rötzsch.</t>
         </is>
@@ -679,7 +712,2161 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:K54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Elemento</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>R4 card.</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>R4 binding/tipo</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>CMD (BRConjuntoMinimoDados-1.1) card.</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>CMD MS</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>CMD binding / fixo / referência</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>br-core-composition 1.3.0 card.</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>br-core-composition MS</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>br-core-composition binding / fixo / referência</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Conformidade CMD × br-core-composition</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Composition.id</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr"/>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr"/>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr"/>
+      <c r="G2" s="5" t="inlineStr"/>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr"/>
+      <c r="J2" s="5" t="inlineStr"/>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Composition.meta</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr"/>
+      <c r="J3" s="5" t="inlineStr"/>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Composition.implicitRules</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr"/>
+      <c r="J4" s="5" t="inlineStr"/>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Composition.language</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>preferred: languages</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>preferred: languages</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr"/>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>preferred: languages</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Composition.text</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr"/>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Composition.contained</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr"/>
+      <c r="J7" s="5" t="inlineStr"/>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Composition.extension</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="5" t="inlineStr"/>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr"/>
+      <c r="J8" s="5" t="inlineStr"/>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Composition.modifierExtension</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr"/>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr"/>
+      <c r="G9" s="5" t="inlineStr"/>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr"/>
+      <c r="J9" s="5" t="inlineStr"/>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Composition.identifier</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>CMD zera o identificador do documento.</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>0..0</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr"/>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr"/>
+      <c r="J10" s="5" t="inlineStr"/>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Composition.status</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>required: composition-status|4.0.1</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>required: BREstadoDocumento-1.0</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr"/>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>required: composition-status</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Composition.type</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>CMD: um único coding, sem display nem text, ValueSet nacional BRTipoDocumento (required). BR-Core: doc-typecodes (preferred).</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>preferred: doc-typecodes</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>required: BRTipoDocumento-1.0</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr"/>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>preferred: doc-typecodes</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Composition.category</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>CMD: modalidade assistencial (BRModalidadeAssistencial, required, 1..1). BR-Core: document-classcodes (example).</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>example: document-classcodes</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>required: BRModalidadeAssistencial-1.0</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr"/>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>example: document-classcodes</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Composition.subject</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>CMD proíbe subject.reference, type e display: o paciente só pode ser identificado por identifier (sistema e valor), ou pela extensão unidentifiedPatient. BR-Core: referência a br-core-patient.</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>ref: Resource</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>ref: BRIndividuo-1.0</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr"/>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>ref: br-core-patient</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Composition.encounter</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>CMD zera encounter; o contato assistencial vira seção obrigatória.</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>ref: Encounter</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>0..0</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr"/>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>ref: Encounter</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr"/>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>ref: br-core-encounter</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Composition.date</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr"/>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr"/>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr"/>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr"/>
+      <c r="J16" s="5" t="inlineStr"/>
+      <c r="K16" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Composition.author</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>CMD proíbe author.reference, type e display e exige identifier: o autor só por identificador. BR-Core: referência a practitioner, practitionerrole, device, organization.</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>1..*</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>ref: Practitioner, PractitionerRole, Device, Patient, RelatedPerson, Organization</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>1..*</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>ref: BRPessoaJuridicaProfissionalLiberal-1.0</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>1..*</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr"/>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>ref: br-core-practitioner, br-core-practitionerrole, Device, br-core-patient, br-core-relatedperson, br-core-organization</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Composition.title</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr"/>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr"/>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr"/>
+      <c r="J18" s="5" t="inlineStr"/>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Composition.confidentiality</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr"/>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>required: v3-ConfidentialityClassification|2014-03-26</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>0..0</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr"/>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>required: v3-ConfidentialityClassification|2014-03-26</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr"/>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>required: v3-ConfidentialityClassification</t>
+        </is>
+      </c>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Composition.attester</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>CMD zera atestação.</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>0..0</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr"/>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr"/>
+      <c r="J20" s="5" t="inlineStr"/>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Composition.attester.id</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr"/>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr"/>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr"/>
+      <c r="G21" s="5" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr"/>
+      <c r="J21" s="5" t="inlineStr"/>
+      <c r="K21" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Composition.attester.extension</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr"/>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr"/>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr"/>
+      <c r="J22" s="5" t="inlineStr"/>
+      <c r="K22" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Composition.attester.modifierExtension</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr"/>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr"/>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr"/>
+      <c r="G23" s="5" t="inlineStr"/>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr"/>
+      <c r="J23" s="5" t="inlineStr"/>
+      <c r="K23" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Composition.attester.mode</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr"/>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>required: composition-attestation-mode|4.0.1</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>required: composition-attestation-mode|4.0.1</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr"/>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>required: composition-attestation-mode</t>
+        </is>
+      </c>
+      <c r="K24" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Composition.attester.time</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr"/>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr"/>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr"/>
+      <c r="G25" s="5" t="inlineStr"/>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr"/>
+      <c r="J25" s="5" t="inlineStr"/>
+      <c r="K25" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Composition.attester.party</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr"/>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>ref: Patient, RelatedPerson, Practitioner, PractitionerRole, Organization</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr"/>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>ref: Patient, RelatedPerson, Practitioner, PractitionerRole, Organization</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr"/>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>ref: br-core-patient, br-core-relatedperson, br-core-practitioner, br-core-practitionerrole, br-core-organization</t>
+        </is>
+      </c>
+      <c r="K26" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Composition.custodian</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>CMD zera custodiante.</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>ref: Organization</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>0..0</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr"/>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>ref: Organization</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr"/>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>ref: br-core-organization</t>
+        </is>
+      </c>
+      <c r="K27" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Composition.relatesTo</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>CMD limita a 1 e exige reference literal.</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr"/>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr"/>
+      <c r="G28" s="5" t="inlineStr"/>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr"/>
+      <c r="J28" s="5" t="inlineStr"/>
+      <c r="K28" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Composition.relatesTo.id</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr"/>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr"/>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr"/>
+      <c r="G29" s="5" t="inlineStr"/>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr"/>
+      <c r="J29" s="5" t="inlineStr"/>
+      <c r="K29" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Composition.relatesTo.extension</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr"/>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr"/>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr"/>
+      <c r="G30" s="5" t="inlineStr"/>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr"/>
+      <c r="J30" s="5" t="inlineStr"/>
+      <c r="K30" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Composition.relatesTo.modifierExtension</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr"/>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr"/>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr"/>
+      <c r="G31" s="5" t="inlineStr"/>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr"/>
+      <c r="J31" s="5" t="inlineStr"/>
+      <c r="K31" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Composition.relatesTo.code</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr"/>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>required: document-relationship-type|4.0.1</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr"/>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>required: document-relationship-type|4.0.1; fixedCode = "replaces"</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr"/>
+      <c r="J32" s="5" t="inlineStr">
+        <is>
+          <t>required: document-relationship-type</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Composition.relatesTo.target[x]</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr"/>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>ref: Composition</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr"/>
+      <c r="G33" s="5" t="inlineStr"/>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>1..1</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr"/>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>ref: Composition; slicing type em $this</t>
+        </is>
+      </c>
+      <c r="K33" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Composition.event</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr"/>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr"/>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>0..0</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr"/>
+      <c r="G34" s="5" t="inlineStr"/>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr"/>
+      <c r="J34" s="5" t="inlineStr"/>
+      <c r="K34" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Composition.event.id</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr"/>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr"/>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr"/>
+      <c r="G35" s="5" t="inlineStr"/>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr"/>
+      <c r="J35" s="5" t="inlineStr"/>
+      <c r="K35" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Composition.event.extension</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr"/>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr"/>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr"/>
+      <c r="G36" s="5" t="inlineStr"/>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr"/>
+      <c r="J36" s="5" t="inlineStr"/>
+      <c r="K36" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Composition.event.modifierExtension</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr"/>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr"/>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr"/>
+      <c r="G37" s="5" t="inlineStr"/>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr"/>
+      <c r="J37" s="5" t="inlineStr"/>
+      <c r="K37" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Composition.event.code</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr"/>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>example: v3-ActCode</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr"/>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>example: v3-ActCode</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr"/>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>required: v3-ActCode</t>
+        </is>
+      </c>
+      <c r="K38" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Composition.event.period</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr"/>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr"/>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr"/>
+      <c r="G39" s="5" t="inlineStr"/>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr"/>
+      <c r="J39" s="5" t="inlineStr"/>
+      <c r="K39" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Composition.event.detail</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr"/>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr"/>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr"/>
+      <c r="G40" s="5" t="inlineStr"/>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr"/>
+      <c r="J40" s="5" t="inlineStr"/>
+      <c r="K40" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Composition.section</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>CMD já fatia as seções (informacoesContatoAssistencial 1..1, problemasDiagnosticosAvaliados, procedimentosRealizados) com code, text e emptyReason zerados. BR-Core não fatia no br-core-composition.</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr"/>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>1..*</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>slicing profile em entry.resolve()</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr"/>
+      <c r="J41" s="5" t="inlineStr"/>
+      <c r="K41" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Composition.section.id</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr"/>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr"/>
+      <c r="G42" s="5" t="inlineStr"/>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr"/>
+      <c r="J42" s="5" t="inlineStr"/>
+      <c r="K42" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Composition.section.extension</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr"/>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr"/>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr"/>
+      <c r="G43" s="5" t="inlineStr"/>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr"/>
+      <c r="J43" s="5" t="inlineStr"/>
+      <c r="K43" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Composition.section.modifierExtension</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr"/>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr"/>
+      <c r="G44" s="5" t="inlineStr"/>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr"/>
+      <c r="J44" s="5" t="inlineStr"/>
+      <c r="K44" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Composition.section.title</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr"/>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr"/>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr"/>
+      <c r="G45" s="5" t="inlineStr"/>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr"/>
+      <c r="J45" s="5" t="inlineStr"/>
+      <c r="K45" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Composition.section.code</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>CMD zera code em todas as suas fatias.</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>example: doc-section-codes</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr"/>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>example: doc-section-codes</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr"/>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>required: doc-section-codes</t>
+        </is>
+      </c>
+      <c r="K46" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Composition.section.author</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr"/>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>ref: Practitioner, PractitionerRole, Device, Patient, RelatedPerson, Organization</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr"/>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>ref: Practitioner, PractitionerRole, Device, Patient, RelatedPerson, Organization</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr"/>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>ref: br-core-practitioner, br-core-practitionerrole, Device, br-core-patient, br-core-relatedperson, br-core-organization</t>
+        </is>
+      </c>
+      <c r="K47" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Composition.section.focus</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr"/>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr"/>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr"/>
+      <c r="G48" s="5" t="inlineStr"/>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr"/>
+      <c r="J48" s="5" t="inlineStr"/>
+      <c r="K48" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Composition.section.text</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>CMD zera text em todas as suas fatias: documento sem narrativa.</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr"/>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr"/>
+      <c r="G49" s="5" t="inlineStr"/>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr"/>
+      <c r="J49" s="5" t="inlineStr"/>
+      <c r="K49" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Composition.section.mode</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr"/>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>required: list-mode|4.0.1</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr"/>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>required: list-mode|4.0.1</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr"/>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>required: list-mode</t>
+        </is>
+      </c>
+      <c r="K50" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Composition.section.orderedBy</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr"/>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>preferred: list-order</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr"/>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>preferred: list-order</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr"/>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>preferred: list-empty-reason</t>
+        </is>
+      </c>
+      <c r="K51" s="6" t="inlineStr">
+        <is>
+          <t>Divergente</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Composition.section.entry</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr"/>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>ref: Resource</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr"/>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>ref: Resource</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr"/>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>ref: Resource</t>
+        </is>
+      </c>
+      <c r="K52" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Composition.section.emptyReason</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr"/>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>preferred: list-empty-reason</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr"/>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>preferred: list-empty-reason</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>0..1</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr"/>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>preferred: list-empty-reason</t>
+        </is>
+      </c>
+      <c r="K53" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Composition.section.section</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr"/>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr"/>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr"/>
+      <c r="G54" s="5" t="inlineStr"/>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>0..*</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr"/>
+      <c r="J54" s="5" t="inlineStr"/>
+      <c r="K54" s="8" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K54"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -698,6 +2885,8 @@
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="60" customWidth="1" min="15" max="15"/>
     <col width="50" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -781,6 +2970,16 @@
           <t>Recomendação</t>
         </is>
       </c>
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
+          <t>Origem da restrição (SA-IG)</t>
+        </is>
+      </c>
+      <c r="R1" s="4" t="inlineStr">
+        <is>
+          <t>Origem da restrição (BR-Core)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -839,6 +3038,16 @@
           <t>Usar identifier (1..1 no documento). Bundle document exige identifier.</t>
         </is>
       </c>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R2" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -913,6 +3122,16 @@
           <t>Usar composition-status do HL7 com suplemento pt-BR (BRSuplementoSituacaoDocumento).</t>
         </is>
       </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>br-core-composition</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -987,6 +3206,16 @@
           <t>LOINC 18842-5 Discharge summary.</t>
         </is>
       </c>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t>br-core-composition</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -1061,6 +3290,16 @@
           <t>Modalidade em Encounter; category = LOINC 107903-7 Clinical note (FHIR Clinical Documents).</t>
         </is>
       </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R5" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1139,6 +3378,16 @@
           <t>br-core-patient.</t>
         </is>
       </c>
+      <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
+          <t>br-core-composition</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1211,6 +3460,16 @@
       <c r="P7" s="5" t="inlineStr">
         <is>
           <t>Composition.encounter para a internação (br-core-encounter); eliminar a seção informacoesContatoAssistencial.</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
+          <t>br-core-composition</t>
         </is>
       </c>
     </row>
@@ -1259,6 +3518,16 @@
       <c r="N8" s="5" t="inlineStr"/>
       <c r="O8" s="5" t="inlineStr"/>
       <c r="P8" s="5" t="inlineStr"/>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1335,6 +3604,16 @@
       <c r="P9" s="5" t="inlineStr">
         <is>
           <t>Perfis do BR-Core.</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>br-core-composition</t>
         </is>
       </c>
     </row>
@@ -1399,6 +3678,16 @@
           <t>Título livre ("Sumário de Alta").</t>
         </is>
       </c>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1471,6 +3760,16 @@
       <c r="P11" s="5" t="inlineStr">
         <is>
           <t>Permitir.</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>br-core-composition</t>
         </is>
       </c>
     </row>
@@ -1531,6 +3830,16 @@
           <t>Atestador legal (FHIR Clinical Documents: attester:legal_attester).</t>
         </is>
       </c>
+      <c r="Q12" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1603,6 +3912,16 @@
       <c r="P13" s="5" t="inlineStr">
         <is>
           <t>Estabelecimento (CNES) como custodian.</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>br-core-composition</t>
         </is>
       </c>
     </row>
@@ -1663,6 +3982,16 @@
           <t>Retificação por relatesTo (replaces).</t>
         </is>
       </c>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R14" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1721,6 +4050,16 @@
           <t>Sem ação.</t>
         </is>
       </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1791,20 +4130,30 @@
           <t>Correção no branch fix/sumarioalta-capacidadefuncional do BR-Core: discriminador pattern em code.</t>
         </is>
       </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R16" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P16"/>
+  <autoFilter ref="A1:R16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P125"/>
+  <dimension ref="A1:R125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1823,6 +4172,8 @@
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="60" customWidth="1" min="15" max="15"/>
     <col width="50" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1906,6 +4257,16 @@
           <t>Recomendação</t>
         </is>
       </c>
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
+          <t>Origem da restrição (SA-IG)</t>
+        </is>
+      </c>
+      <c r="R1" s="4" t="inlineStr">
+        <is>
+          <t>Origem da restrição (BR-Core)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -1964,6 +4325,16 @@
           <t>Eliminar a seção; usar Composition.encounter.</t>
         </is>
       </c>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R2" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -2026,6 +4397,16 @@
           <t>Título livre.</t>
         </is>
       </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -2092,6 +4473,16 @@
           <t>Código LOINC por seção.</t>
         </is>
       </c>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -2150,6 +4541,16 @@
           <t>Narrativa em section.text (FHIR Clinical Documents exige).</t>
         </is>
       </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R5" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -2204,6 +4605,16 @@
       <c r="N6" s="5" t="inlineStr"/>
       <c r="O6" s="5" t="inlineStr"/>
       <c r="P6" s="5" t="inlineStr"/>
+      <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2258,6 +4669,16 @@
       <c r="N7" s="5" t="inlineStr"/>
       <c r="O7" s="5" t="inlineStr"/>
       <c r="P7" s="5" t="inlineStr"/>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -2324,6 +4745,16 @@
           <t>Várias entradas na mesma seção.</t>
         </is>
       </c>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -2390,6 +4821,16 @@
           <t>Usar emptyReason (list-empty-reason).</t>
         </is>
       </c>
+      <c r="Q9" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -2444,6 +4885,16 @@
       <c r="N10" s="5" t="inlineStr"/>
       <c r="O10" s="5" t="inlineStr"/>
       <c r="P10" s="5" t="inlineStr"/>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -2490,6 +4941,16 @@
       <c r="N11" s="5" t="inlineStr"/>
       <c r="O11" s="5" t="inlineStr"/>
       <c r="P11" s="5" t="inlineStr"/>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -2536,6 +4997,16 @@
       <c r="N12" s="5" t="inlineStr"/>
       <c r="O12" s="5" t="inlineStr"/>
       <c r="P12" s="5" t="inlineStr"/>
+      <c r="Q12" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -2598,6 +5069,16 @@
           <t>Separar em duas seções.</t>
         </is>
       </c>
+      <c r="Q13" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -2660,6 +5141,16 @@
           <t>Título livre.</t>
         </is>
       </c>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R14" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -2734,6 +5225,16 @@
           <t>Código LOINC por seção.</t>
         </is>
       </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -2798,6 +5299,16 @@
       <c r="P16" s="5" t="inlineStr">
         <is>
           <t>Corrigido no branch: http://loinc.org.</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R16" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
         </is>
       </c>
     </row>
@@ -2854,6 +5365,16 @@
       <c r="N17" s="5" t="inlineStr"/>
       <c r="O17" s="5" t="inlineStr"/>
       <c r="P17" s="5" t="inlineStr"/>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -2912,6 +5433,16 @@
           <t>Narrativa em section.text (FHIR Clinical Documents exige).</t>
         </is>
       </c>
+      <c r="Q18" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R18" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -2974,6 +5505,16 @@
       <c r="N19" s="5" t="inlineStr"/>
       <c r="O19" s="5" t="inlineStr"/>
       <c r="P19" s="5" t="inlineStr"/>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -3036,6 +5577,16 @@
       <c r="N20" s="5" t="inlineStr"/>
       <c r="O20" s="5" t="inlineStr"/>
       <c r="P20" s="5" t="inlineStr"/>
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -3110,6 +5661,16 @@
           <t>Várias entradas na mesma seção.</t>
         </is>
       </c>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -3182,6 +5743,16 @@
       <c r="P22" s="5" t="inlineStr">
         <is>
           <t>Usar emptyReason (list-empty-reason).</t>
+        </is>
+      </c>
+      <c r="Q22" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R22" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
         </is>
       </c>
     </row>
@@ -3246,6 +5817,16 @@
       <c r="N23" s="5" t="inlineStr"/>
       <c r="O23" s="5" t="inlineStr"/>
       <c r="P23" s="5" t="inlineStr"/>
+      <c r="Q23" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R23" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -3292,6 +5873,16 @@
       <c r="N24" s="5" t="inlineStr"/>
       <c r="O24" s="5" t="inlineStr"/>
       <c r="P24" s="5" t="inlineStr"/>
+      <c r="Q24" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R24" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -3338,6 +5929,16 @@
       <c r="N25" s="5" t="inlineStr"/>
       <c r="O25" s="5" t="inlineStr"/>
       <c r="P25" s="5" t="inlineStr"/>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -3400,6 +6001,16 @@
           <t>Separar em duas seções.</t>
         </is>
       </c>
+      <c r="Q26" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R26" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -3462,6 +6073,16 @@
           <t>Título livre.</t>
         </is>
       </c>
+      <c r="Q27" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R27" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -3536,6 +6157,16 @@
           <t>Código LOINC por seção.</t>
         </is>
       </c>
+      <c r="Q28" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R28" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -3600,6 +6231,16 @@
       <c r="P29" s="5" t="inlineStr">
         <is>
           <t>Corrigido no branch: http://loinc.org.</t>
+        </is>
+      </c>
+      <c r="Q29" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R29" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
         </is>
       </c>
     </row>
@@ -3656,6 +6297,16 @@
       <c r="N30" s="5" t="inlineStr"/>
       <c r="O30" s="5" t="inlineStr"/>
       <c r="P30" s="5" t="inlineStr"/>
+      <c r="Q30" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R30" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -3714,6 +6365,16 @@
           <t>Narrativa em section.text (FHIR Clinical Documents exige).</t>
         </is>
       </c>
+      <c r="Q31" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R31" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -3776,6 +6437,16 @@
       <c r="N32" s="5" t="inlineStr"/>
       <c r="O32" s="5" t="inlineStr"/>
       <c r="P32" s="5" t="inlineStr"/>
+      <c r="Q32" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R32" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -3838,6 +6509,16 @@
       <c r="N33" s="5" t="inlineStr"/>
       <c r="O33" s="5" t="inlineStr"/>
       <c r="P33" s="5" t="inlineStr"/>
+      <c r="Q33" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R33" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -3912,6 +6593,16 @@
           <t>Várias entradas na mesma seção.</t>
         </is>
       </c>
+      <c r="Q34" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R34" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -3984,6 +6675,16 @@
       <c r="P35" s="5" t="inlineStr">
         <is>
           <t>Usar emptyReason (list-empty-reason).</t>
+        </is>
+      </c>
+      <c r="Q35" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R35" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
         </is>
       </c>
     </row>
@@ -4048,6 +6749,16 @@
       <c r="N36" s="5" t="inlineStr"/>
       <c r="O36" s="5" t="inlineStr"/>
       <c r="P36" s="5" t="inlineStr"/>
+      <c r="Q36" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R36" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -4094,6 +6805,16 @@
       <c r="N37" s="5" t="inlineStr"/>
       <c r="O37" s="5" t="inlineStr"/>
       <c r="P37" s="5" t="inlineStr"/>
+      <c r="Q37" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R37" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -4140,6 +6861,16 @@
       <c r="N38" s="5" t="inlineStr"/>
       <c r="O38" s="5" t="inlineStr"/>
       <c r="P38" s="5" t="inlineStr"/>
+      <c r="Q38" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R38" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -4198,6 +6929,16 @@
           <t>Seção única com emptyReason quando não houver alergias.</t>
         </is>
       </c>
+      <c r="Q39" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
+      <c r="R39" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -4260,6 +7001,16 @@
           <t>Título livre.</t>
         </is>
       </c>
+      <c r="Q40" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R40" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
@@ -4334,6 +7085,16 @@
           <t>Código LOINC por seção.</t>
         </is>
       </c>
+      <c r="Q41" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R41" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -4398,6 +7159,16 @@
       <c r="P42" s="5" t="inlineStr">
         <is>
           <t>Corrigido no branch: http://loinc.org.</t>
+        </is>
+      </c>
+      <c r="Q42" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R42" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
         </is>
       </c>
     </row>
@@ -4454,6 +7225,16 @@
       <c r="N43" s="5" t="inlineStr"/>
       <c r="O43" s="5" t="inlineStr"/>
       <c r="P43" s="5" t="inlineStr"/>
+      <c r="Q43" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R43" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -4512,6 +7293,16 @@
           <t>Narrativa em section.text (FHIR Clinical Documents exige).</t>
         </is>
       </c>
+      <c r="Q44" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R44" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -4574,6 +7365,16 @@
       <c r="N45" s="5" t="inlineStr"/>
       <c r="O45" s="5" t="inlineStr"/>
       <c r="P45" s="5" t="inlineStr"/>
+      <c r="Q45" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R45" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -4636,6 +7437,16 @@
       <c r="N46" s="5" t="inlineStr"/>
       <c r="O46" s="5" t="inlineStr"/>
       <c r="P46" s="5" t="inlineStr"/>
+      <c r="Q46" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R46" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -4710,6 +7521,16 @@
           <t>Várias entradas na mesma seção.</t>
         </is>
       </c>
+      <c r="Q47" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R47" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -4782,6 +7603,16 @@
       <c r="P48" s="5" t="inlineStr">
         <is>
           <t>Usar emptyReason (list-empty-reason).</t>
+        </is>
+      </c>
+      <c r="Q48" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R48" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
         </is>
       </c>
     </row>
@@ -4846,6 +7677,16 @@
       <c r="N49" s="5" t="inlineStr"/>
       <c r="O49" s="5" t="inlineStr"/>
       <c r="P49" s="5" t="inlineStr"/>
+      <c r="Q49" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R49" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
@@ -4892,6 +7733,16 @@
       <c r="N50" s="5" t="inlineStr"/>
       <c r="O50" s="5" t="inlineStr"/>
       <c r="P50" s="5" t="inlineStr"/>
+      <c r="Q50" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R50" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
@@ -4938,6 +7789,16 @@
       <c r="N51" s="5" t="inlineStr"/>
       <c r="O51" s="5" t="inlineStr"/>
       <c r="P51" s="5" t="inlineStr"/>
+      <c r="Q51" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R51" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -4996,6 +7857,16 @@
           <t>Uma seção com várias entradas.</t>
         </is>
       </c>
+      <c r="Q52" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R52" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
@@ -5058,6 +7929,16 @@
           <t>Título livre.</t>
         </is>
       </c>
+      <c r="Q53" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R53" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
@@ -5132,6 +8013,16 @@
           <t>Código LOINC por seção.</t>
         </is>
       </c>
+      <c r="Q54" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R54" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
@@ -5196,6 +8087,16 @@
       <c r="P55" s="5" t="inlineStr">
         <is>
           <t>Corrigido no branch: http://loinc.org.</t>
+        </is>
+      </c>
+      <c r="Q55" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R55" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
         </is>
       </c>
     </row>
@@ -5252,6 +8153,16 @@
       <c r="N56" s="5" t="inlineStr"/>
       <c r="O56" s="5" t="inlineStr"/>
       <c r="P56" s="5" t="inlineStr"/>
+      <c r="Q56" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R56" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
@@ -5310,6 +8221,16 @@
           <t>Narrativa em section.text (FHIR Clinical Documents exige).</t>
         </is>
       </c>
+      <c r="Q57" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R57" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
@@ -5372,6 +8293,16 @@
       <c r="N58" s="5" t="inlineStr"/>
       <c r="O58" s="5" t="inlineStr"/>
       <c r="P58" s="5" t="inlineStr"/>
+      <c r="Q58" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R58" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
@@ -5434,6 +8365,16 @@
       <c r="N59" s="5" t="inlineStr"/>
       <c r="O59" s="5" t="inlineStr"/>
       <c r="P59" s="5" t="inlineStr"/>
+      <c r="Q59" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R59" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
@@ -5508,6 +8449,16 @@
           <t>Várias entradas na mesma seção.</t>
         </is>
       </c>
+      <c r="Q60" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R60" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
@@ -5580,6 +8531,16 @@
       <c r="P61" s="5" t="inlineStr">
         <is>
           <t>Usar emptyReason (list-empty-reason).</t>
+        </is>
+      </c>
+      <c r="Q61" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R61" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
         </is>
       </c>
     </row>
@@ -5644,6 +8605,16 @@
       <c r="N62" s="5" t="inlineStr"/>
       <c r="O62" s="5" t="inlineStr"/>
       <c r="P62" s="5" t="inlineStr"/>
+      <c r="Q62" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R62" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
@@ -5690,6 +8661,16 @@
       <c r="N63" s="5" t="inlineStr"/>
       <c r="O63" s="5" t="inlineStr"/>
       <c r="P63" s="5" t="inlineStr"/>
+      <c r="Q63" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R63" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -5736,6 +8717,16 @@
       <c r="N64" s="5" t="inlineStr"/>
       <c r="O64" s="5" t="inlineStr"/>
       <c r="P64" s="5" t="inlineStr"/>
+      <c r="Q64" s="5" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="R64" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
@@ -5794,6 +8785,16 @@
           <t>Entradas diretamente em MedicationRequest.</t>
         </is>
       </c>
+      <c r="Q65" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R65" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
@@ -5856,6 +8857,16 @@
           <t>Título livre.</t>
         </is>
       </c>
+      <c r="Q66" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R66" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
@@ -5930,6 +8941,16 @@
           <t>Código LOINC por seção.</t>
         </is>
       </c>
+      <c r="Q67" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R67" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
@@ -5994,6 +9015,16 @@
       <c r="P68" s="5" t="inlineStr">
         <is>
           <t>Corrigido no branch: http://loinc.org.</t>
+        </is>
+      </c>
+      <c r="Q68" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R68" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
         </is>
       </c>
     </row>
@@ -6050,6 +9081,16 @@
       <c r="N69" s="5" t="inlineStr"/>
       <c r="O69" s="5" t="inlineStr"/>
       <c r="P69" s="5" t="inlineStr"/>
+      <c r="Q69" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R69" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
@@ -6108,6 +9149,16 @@
           <t>Narrativa em section.text (FHIR Clinical Documents exige).</t>
         </is>
       </c>
+      <c r="Q70" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R70" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
@@ -6170,6 +9221,16 @@
       <c r="N71" s="5" t="inlineStr"/>
       <c r="O71" s="5" t="inlineStr"/>
       <c r="P71" s="5" t="inlineStr"/>
+      <c r="Q71" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R71" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
@@ -6232,6 +9293,16 @@
       <c r="N72" s="5" t="inlineStr"/>
       <c r="O72" s="5" t="inlineStr"/>
       <c r="P72" s="5" t="inlineStr"/>
+      <c r="Q72" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R72" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
@@ -6306,6 +9377,16 @@
           <t>Várias entradas na mesma seção.</t>
         </is>
       </c>
+      <c r="Q73" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R73" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
@@ -6378,6 +9459,16 @@
       <c r="P74" s="5" t="inlineStr">
         <is>
           <t>Usar emptyReason (list-empty-reason).</t>
+        </is>
+      </c>
+      <c r="Q74" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R74" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
         </is>
       </c>
     </row>
@@ -6442,6 +9533,16 @@
       <c r="N75" s="5" t="inlineStr"/>
       <c r="O75" s="5" t="inlineStr"/>
       <c r="P75" s="5" t="inlineStr"/>
+      <c r="Q75" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R75" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
@@ -6488,6 +9589,16 @@
       <c r="N76" s="5" t="inlineStr"/>
       <c r="O76" s="5" t="inlineStr"/>
       <c r="P76" s="5" t="inlineStr"/>
+      <c r="Q76" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R76" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
@@ -6534,6 +9645,16 @@
       <c r="N77" s="5" t="inlineStr"/>
       <c r="O77" s="5" t="inlineStr"/>
       <c r="P77" s="5" t="inlineStr"/>
+      <c r="Q77" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R77" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
@@ -6592,6 +9713,16 @@
           <t>br-core-careplan.</t>
         </is>
       </c>
+      <c r="Q78" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R78" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
@@ -6654,6 +9785,16 @@
           <t>Título livre.</t>
         </is>
       </c>
+      <c r="Q79" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R79" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
@@ -6728,6 +9869,16 @@
           <t>Código LOINC por seção.</t>
         </is>
       </c>
+      <c r="Q80" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R80" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
@@ -6792,6 +9943,16 @@
       <c r="P81" s="5" t="inlineStr">
         <is>
           <t>Corrigido no branch: http://loinc.org.</t>
+        </is>
+      </c>
+      <c r="Q81" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R81" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
         </is>
       </c>
     </row>
@@ -6848,6 +10009,16 @@
       <c r="N82" s="5" t="inlineStr"/>
       <c r="O82" s="5" t="inlineStr"/>
       <c r="P82" s="5" t="inlineStr"/>
+      <c r="Q82" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R82" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
@@ -6906,6 +10077,16 @@
           <t>Narrativa em section.text (FHIR Clinical Documents exige).</t>
         </is>
       </c>
+      <c r="Q83" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R83" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
@@ -6968,6 +10149,16 @@
       <c r="N84" s="5" t="inlineStr"/>
       <c r="O84" s="5" t="inlineStr"/>
       <c r="P84" s="5" t="inlineStr"/>
+      <c r="Q84" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R84" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
@@ -7030,6 +10221,16 @@
       <c r="N85" s="5" t="inlineStr"/>
       <c r="O85" s="5" t="inlineStr"/>
       <c r="P85" s="5" t="inlineStr"/>
+      <c r="Q85" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R85" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
@@ -7104,6 +10305,16 @@
           <t>Várias entradas na mesma seção.</t>
         </is>
       </c>
+      <c r="Q86" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R86" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
@@ -7176,6 +10387,16 @@
       <c r="P87" s="5" t="inlineStr">
         <is>
           <t>Usar emptyReason (list-empty-reason).</t>
+        </is>
+      </c>
+      <c r="Q87" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R87" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
         </is>
       </c>
     </row>
@@ -7240,6 +10461,16 @@
       <c r="N88" s="5" t="inlineStr"/>
       <c r="O88" s="5" t="inlineStr"/>
       <c r="P88" s="5" t="inlineStr"/>
+      <c r="Q88" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R88" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
@@ -7286,6 +10517,16 @@
       <c r="N89" s="5" t="inlineStr"/>
       <c r="O89" s="5" t="inlineStr"/>
       <c r="P89" s="5" t="inlineStr"/>
+      <c r="Q89" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R89" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
@@ -7332,6 +10573,16 @@
       <c r="N90" s="5" t="inlineStr"/>
       <c r="O90" s="5" t="inlineStr"/>
       <c r="P90" s="5" t="inlineStr"/>
+      <c r="Q90" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R90" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
@@ -7390,6 +10641,16 @@
           <t>br-core-capacidadefuncional (correção no branch).</t>
         </is>
       </c>
+      <c r="Q91" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R91" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
@@ -7452,6 +10713,16 @@
           <t>Título livre.</t>
         </is>
       </c>
+      <c r="Q92" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R92" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
@@ -7526,6 +10797,16 @@
           <t>Código LOINC por seção.</t>
         </is>
       </c>
+      <c r="Q93" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R93" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
@@ -7590,6 +10871,16 @@
       <c r="P94" s="5" t="inlineStr">
         <is>
           <t>Corrigido no branch: http://loinc.org.</t>
+        </is>
+      </c>
+      <c r="Q94" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R94" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
         </is>
       </c>
     </row>
@@ -7646,6 +10937,16 @@
       <c r="N95" s="5" t="inlineStr"/>
       <c r="O95" s="5" t="inlineStr"/>
       <c r="P95" s="5" t="inlineStr"/>
+      <c r="Q95" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R95" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
@@ -7704,6 +11005,16 @@
           <t>Narrativa em section.text (FHIR Clinical Documents exige).</t>
         </is>
       </c>
+      <c r="Q96" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R96" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
@@ -7766,6 +11077,16 @@
       <c r="N97" s="5" t="inlineStr"/>
       <c r="O97" s="5" t="inlineStr"/>
       <c r="P97" s="5" t="inlineStr"/>
+      <c r="Q97" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R97" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
@@ -7828,6 +11149,16 @@
       <c r="N98" s="5" t="inlineStr"/>
       <c r="O98" s="5" t="inlineStr"/>
       <c r="P98" s="5" t="inlineStr"/>
+      <c r="Q98" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R98" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
@@ -7902,6 +11233,16 @@
           <t>Várias entradas na mesma seção.</t>
         </is>
       </c>
+      <c r="Q99" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R99" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
@@ -7974,6 +11315,16 @@
       <c r="P100" s="5" t="inlineStr">
         <is>
           <t>Usar emptyReason (list-empty-reason).</t>
+        </is>
+      </c>
+      <c r="Q100" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R100" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
         </is>
       </c>
     </row>
@@ -8038,6 +11389,16 @@
       <c r="N101" s="5" t="inlineStr"/>
       <c r="O101" s="5" t="inlineStr"/>
       <c r="P101" s="5" t="inlineStr"/>
+      <c r="Q101" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R101" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
@@ -8084,6 +11445,16 @@
       <c r="N102" s="5" t="inlineStr"/>
       <c r="O102" s="5" t="inlineStr"/>
       <c r="P102" s="5" t="inlineStr"/>
+      <c r="Q102" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R102" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
@@ -8130,6 +11501,16 @@
       <c r="N103" s="5" t="inlineStr"/>
       <c r="O103" s="5" t="inlineStr"/>
       <c r="P103" s="5" t="inlineStr"/>
+      <c r="Q103" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R103" s="5" t="inlineStr">
+        <is>
+          <t>Composition (R4)</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
@@ -8188,6 +11569,16 @@
           <t>Encounter.text (resumo da evolução).</t>
         </is>
       </c>
+      <c r="Q104" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R104" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
@@ -8250,6 +11641,16 @@
           <t>Título livre.</t>
         </is>
       </c>
+      <c r="Q105" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R105" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
@@ -8316,6 +11717,16 @@
           <t>Código LOINC por seção.</t>
         </is>
       </c>
+      <c r="Q106" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R106" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
@@ -8374,6 +11785,16 @@
           <t>Narrativa em section.text (FHIR Clinical Documents exige).</t>
         </is>
       </c>
+      <c r="Q107" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R107" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
@@ -8428,6 +11849,16 @@
       <c r="N108" s="5" t="inlineStr"/>
       <c r="O108" s="5" t="inlineStr"/>
       <c r="P108" s="5" t="inlineStr"/>
+      <c r="Q108" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R108" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
@@ -8482,6 +11913,16 @@
       <c r="N109" s="5" t="inlineStr"/>
       <c r="O109" s="5" t="inlineStr"/>
       <c r="P109" s="5" t="inlineStr"/>
+      <c r="Q109" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R109" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
@@ -8548,6 +11989,16 @@
           <t>Várias entradas na mesma seção.</t>
         </is>
       </c>
+      <c r="Q110" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R110" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
@@ -8614,6 +12065,16 @@
           <t>Usar emptyReason (list-empty-reason).</t>
         </is>
       </c>
+      <c r="Q111" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R111" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
@@ -8668,6 +12129,16 @@
       <c r="N112" s="5" t="inlineStr"/>
       <c r="O112" s="5" t="inlineStr"/>
       <c r="P112" s="5" t="inlineStr"/>
+      <c r="Q112" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R112" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
@@ -8714,6 +12185,16 @@
       <c r="N113" s="5" t="inlineStr"/>
       <c r="O113" s="5" t="inlineStr"/>
       <c r="P113" s="5" t="inlineStr"/>
+      <c r="Q113" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R113" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
@@ -8760,6 +12241,16 @@
       <c r="N114" s="5" t="inlineStr"/>
       <c r="O114" s="5" t="inlineStr"/>
       <c r="P114" s="5" t="inlineStr"/>
+      <c r="Q114" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R114" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
@@ -8818,6 +12309,16 @@
           <t>Levar para o Encounter ou para section.text.</t>
         </is>
       </c>
+      <c r="Q115" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R115" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
@@ -8880,6 +12381,16 @@
           <t>Título livre.</t>
         </is>
       </c>
+      <c r="Q116" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R116" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
@@ -8946,6 +12457,16 @@
           <t>Código LOINC por seção.</t>
         </is>
       </c>
+      <c r="Q117" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R117" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
@@ -9004,6 +12525,16 @@
           <t>Narrativa em section.text (FHIR Clinical Documents exige).</t>
         </is>
       </c>
+      <c r="Q118" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R118" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
@@ -9058,6 +12589,16 @@
       <c r="N119" s="5" t="inlineStr"/>
       <c r="O119" s="5" t="inlineStr"/>
       <c r="P119" s="5" t="inlineStr"/>
+      <c r="Q119" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R119" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
@@ -9112,6 +12653,16 @@
       <c r="N120" s="5" t="inlineStr"/>
       <c r="O120" s="5" t="inlineStr"/>
       <c r="P120" s="5" t="inlineStr"/>
+      <c r="Q120" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R120" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
@@ -9178,6 +12729,16 @@
           <t>Várias entradas na mesma seção.</t>
         </is>
       </c>
+      <c r="Q121" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R121" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
@@ -9244,6 +12805,16 @@
           <t>Usar emptyReason (list-empty-reason).</t>
         </is>
       </c>
+      <c r="Q122" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R122" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
@@ -9298,6 +12869,16 @@
       <c r="N123" s="5" t="inlineStr"/>
       <c r="O123" s="5" t="inlineStr"/>
       <c r="P123" s="5" t="inlineStr"/>
+      <c r="Q123" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R123" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
@@ -9344,6 +12925,16 @@
       <c r="N124" s="5" t="inlineStr"/>
       <c r="O124" s="5" t="inlineStr"/>
       <c r="P124" s="5" t="inlineStr"/>
+      <c r="Q124" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R124" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
@@ -9390,14 +12981,24 @@
       <c r="N125" s="5" t="inlineStr"/>
       <c r="O125" s="5" t="inlineStr"/>
       <c r="P125" s="5" t="inlineStr"/>
+      <c r="Q125" s="5" t="inlineStr">
+        <is>
+          <t>BRSumarioAlta</t>
+        </is>
+      </c>
+      <c r="R125" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P125"/>
+  <autoFilter ref="A1:R125"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
comparativo: cotejo com comparativo_sa.xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UVSEtwhqSH6xEBzE8dBMwP
</commit_message>
<xml_diff>
--- a/comparativo/comparativo_sumarioalta_rnds_brcore.xlsx
+++ b/comparativo/comparativo_sumarioalta_rnds_brcore.xlsx
@@ -8,16 +8,17 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CMD × br-core-composition" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composition" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seções" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Débitos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cotejo com comparativo_sa" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CMD × br-core-composition" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Composition" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seções" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Débitos" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CMD × br-core-composition'!$A$1:$K$54</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Composition'!$A$1:$R$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Seções'!$A$1:$R$125</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Débitos'!$A$1:$E$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CMD × br-core-composition'!$A$1:$K$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Composition'!$A$1:$R$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Seções'!$A$1:$R$125</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Débitos'!$A$1:$E$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -59,7 +60,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -96,6 +97,16 @@
         <fgColor rgb="00EFEFEF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CFE2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAD1DC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -123,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -153,6 +164,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -712,6 +732,520 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>comparativo_sa.xlsx (anterior)</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Este comparativo</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Situação</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>Encaminhamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Fontes</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>SA-IG em JSON × FSH do BR-Core (código-fonte do repositório). Sem coluna R4 (declarado no Leia-me).</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>SA-IG em snapshot × pacote BR-Core 1.3.0 em snapshot × R4 × BR-Core corrigido (branch).</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Divergem no método</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Snapshot mostra o que o validador usa; o FSH não mostra herança nem o efeito do alias $loinc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Escopo</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Seções do documento, cinco recursos clínicos (Condition, AllergyIntolerance, Procedure, MedicationRequest, CarePlan) e inventário dos 24 perfis.</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Cabeçalho da Composition, seções e subelementos, e o nível CMD × br-core-composition.</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Complementares</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Usar os dois: o anterior para os recursos clínicos, este para o documento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Camada CMD</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Cita que BRSumarioAlta deriva do CMD e que o CMD zera encounter.</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Compara o CMD com o br-core-composition elemento a elemento e indica a origem de cada restrição.</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Só neste</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>A maior parte das restrições do cabeçalho vem do CMD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Cabeçalho da Composition</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Não compara (só encounter).</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>identifier, attester, custodian e confidentiality proibidos; title fixo "Conjunto Mínimo de Dados"; status em ValueSet nacional; category usada para modalidade; subject e author só por identificador.</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Só neste</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Incluir nos débitos do SA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Cardinalidade das seções no SA-IG</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>"Nenhuma das 9 seções tem cardinalidade total fixa"; procedimentosRealizados sem cardinalidade.</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>section 1..*; informacoesContatoAssistencial 1..1; procedimentosRealizados 1..*; resumoEvolucaoClinica 1..1 (snapshot).</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Divergem</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>O anterior leu só o differential do BRSumarioAlta; o mínimo vem do CMD e aparece no snapshot. Procedimentos é obrigatório no SA-IG.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Fatiamento das seções no SA-IG</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Não registra.</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Discriminador profile em entry.resolve(); cada seção leva uma entrada e se repete.</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Só neste</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>section.code, section.text e emptyReason no SA-IG</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Não registra.</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Os três proibidos (0..0) em todas as seções: sem código, sem narrativa, sem justificativa de seção vazia.</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Só neste</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Com o BR-Core corrigido, seção sem code não casa com nenhuma fatia: bloqueante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>br-core-sumarioalta: discriminador e sistema LOINC</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Descreve os códigos como "fixos" e recomenda migrar para Parent br-core-sumarioalta.</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Discriminador profile em code e system https://loinc.org/: nenhuma instância valida (D-01, D-02). Corrigido no branch.</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Divergem</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>A recomendação anterior só é viável depois da correção do BR-Core.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Seções 9 → 7</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Mesma correspondência: contato e informações adicionais sem seção; diagnósticos desdobrados; capacidade funcional obrigatória.</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Mesma correspondência.</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Concordam</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Grau: contato assistencial e resumo da evolução</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Médio e Médio.</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Alto e Alto.</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Divergem no grau</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Ambos zeram/recriam elementos nativos (encounter, Encounter.text); tratado como Alto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Paciente não identificado</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Recomenda CNS provisório no lugar da extensão unidentifiedPatient.</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Concorda e acrescenta que o br-core-patient exige CPF (1..1), o que impede o CNS provisório (D-03).</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Este completa</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Decisão pendente no BR-Core.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Procedure.code</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Recompor com SIGTAP, TUSS-22 e CBHPM.</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>BRProcedimentosNacionais com BRTabelaSUS e TUSS 22; CBHPM fora (AMB, paga).</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>Superado por decisão</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Decisão de 02/10/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Capacidade funcional</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Remodelar sobre br-core-condition com ValueSet nacional de capacidade funcional.</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>br-core-capacidadefuncional corrigido: SNOMED CT Functional finding (BRCapacidadeFuncional), CID-10 adicional, sem subject.identifier e stage obrigatórios.</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Superado por decisão</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Correção no branch do BR-Core.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Alergias e manifestações</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>SNOMED CT (GPS) no lugar de BRAlergenos/MedDRA.</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>SNOMED CT + CBARA (152 códigos mapeados no OCL) e MedDRA mapeado (28).</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Este completa</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Perfil próprio do SA</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Recomenda migrar BRSumarioAlta para Parent br-core-sumarioalta.</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Sem perfil próprio: usa br-core-sumarioalta direto; regras viram preenchimento e propostas ao BR-Core.</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Superado por decisão</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>A RNDS se ajusta ao BR-Core.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Bundle do documento</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Não trata.</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>br-core-bundle-documento criado no branch; segue o clinical-document-bundle.</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Só neste</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Recursos clínicos (Condition, AllergyIntolerance, Procedure, MedicationRequest, CarePlan)</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Comparação elemento a elemento com débito e recomendação.</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Não repete.</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Só no anterior</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Continua válido; atualizar Procedure.code e capacidade funcional conforme decisões.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Inventário de perfis do SA-IG</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>24 perfis com versão, data e equivalente no BR-Core.</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Não repete.</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Só no anterior</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2860,7 +3394,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4147,7 +4681,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12998,7 +13532,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs: mapa de estrutura, modelo lógico e índice com motivo e método da refatoração
- Página Mapa de estrutura (substitui Comparativos), gerada da planilha e do modelo lógico
- Modelo lógico SumarioAltaML com mapeamentos para BR-Core e SA-IG
- Índice: por que refatorar e como foi feito
- D-02 reescrito: ValueSet doc-section-codes, CodeSystem LOINC (http://loinc.org)
- D-38 (SA-IG sem modelo lógico) e D-39 (códigos de seção fora do doc-section-codes)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UVSEtwhqSH6xEBzE8dBMwP
</commit_message>
<xml_diff>
--- a/comparativo/comparativo_sumarioalta_rnds_brcore.xlsx
+++ b/comparativo/comparativo_sumarioalta_rnds_brcore.xlsx
@@ -5827,7 +5827,7 @@
       </c>
       <c r="O16" s="5" t="inlineStr">
         <is>
-          <t>BR-Core 1.3.0 fixa https://loinc.org/, rejeitado pelo binding required doc-section-codes.</t>
+          <t>BR-Core 1.3.0 fixa https://loinc.org/. O binding é o ValueSet doc-section-codes (required), com códigos do CodeSystem LOINC, de canonical http://loinc.org; com https://loinc.org/ o código não pertence ao ValueSet.</t>
         </is>
       </c>
       <c r="P16" s="5" t="inlineStr">
@@ -6759,7 +6759,7 @@
       </c>
       <c r="O29" s="5" t="inlineStr">
         <is>
-          <t>BR-Core 1.3.0 fixa https://loinc.org/, rejeitado pelo binding required doc-section-codes.</t>
+          <t>BR-Core 1.3.0 fixa https://loinc.org/. O binding é o ValueSet doc-section-codes (required), com códigos do CodeSystem LOINC, de canonical http://loinc.org; com https://loinc.org/ o código não pertence ao ValueSet.</t>
         </is>
       </c>
       <c r="P29" s="5" t="inlineStr">
@@ -7687,7 +7687,7 @@
       </c>
       <c r="O42" s="5" t="inlineStr">
         <is>
-          <t>BR-Core 1.3.0 fixa https://loinc.org/, rejeitado pelo binding required doc-section-codes.</t>
+          <t>BR-Core 1.3.0 fixa https://loinc.org/. O binding é o ValueSet doc-section-codes (required), com códigos do CodeSystem LOINC, de canonical http://loinc.org; com https://loinc.org/ o código não pertence ao ValueSet.</t>
         </is>
       </c>
       <c r="P42" s="5" t="inlineStr">
@@ -8615,7 +8615,7 @@
       </c>
       <c r="O55" s="5" t="inlineStr">
         <is>
-          <t>BR-Core 1.3.0 fixa https://loinc.org/, rejeitado pelo binding required doc-section-codes.</t>
+          <t>BR-Core 1.3.0 fixa https://loinc.org/. O binding é o ValueSet doc-section-codes (required), com códigos do CodeSystem LOINC, de canonical http://loinc.org; com https://loinc.org/ o código não pertence ao ValueSet.</t>
         </is>
       </c>
       <c r="P55" s="5" t="inlineStr">
@@ -9543,7 +9543,7 @@
       </c>
       <c r="O68" s="5" t="inlineStr">
         <is>
-          <t>BR-Core 1.3.0 fixa https://loinc.org/, rejeitado pelo binding required doc-section-codes.</t>
+          <t>BR-Core 1.3.0 fixa https://loinc.org/. O binding é o ValueSet doc-section-codes (required), com códigos do CodeSystem LOINC, de canonical http://loinc.org; com https://loinc.org/ o código não pertence ao ValueSet.</t>
         </is>
       </c>
       <c r="P68" s="5" t="inlineStr">
@@ -10471,7 +10471,7 @@
       </c>
       <c r="O81" s="5" t="inlineStr">
         <is>
-          <t>BR-Core 1.3.0 fixa https://loinc.org/, rejeitado pelo binding required doc-section-codes.</t>
+          <t>BR-Core 1.3.0 fixa https://loinc.org/. O binding é o ValueSet doc-section-codes (required), com códigos do CodeSystem LOINC, de canonical http://loinc.org; com https://loinc.org/ o código não pertence ao ValueSet.</t>
         </is>
       </c>
       <c r="P81" s="5" t="inlineStr">
@@ -11399,7 +11399,7 @@
       </c>
       <c r="O94" s="5" t="inlineStr">
         <is>
-          <t>BR-Core 1.3.0 fixa https://loinc.org/, rejeitado pelo binding required doc-section-codes.</t>
+          <t>BR-Core 1.3.0 fixa https://loinc.org/. O binding é o ValueSet doc-section-codes (required), com códigos do CodeSystem LOINC, de canonical http://loinc.org; com https://loinc.org/ o código não pertence ao ValueSet.</t>
         </is>
       </c>
       <c r="P94" s="5" t="inlineStr">
@@ -13538,7 +13538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -13647,7 +13647,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>BR-Core 1.3.0 fixa https://loinc.org/, rejeitado pelo binding required doc-section-codes.</t>
+          <t>BR-Core 1.3.0 fixa https://loinc.org/. O binding é o ValueSet doc-section-codes (required), com códigos do CodeSystem LOINC, de canonical http://loinc.org; com https://loinc.org/ o código não pertence ao ValueSet.</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -14382,6 +14382,33 @@
       <c r="E31" s="5" t="inlineStr">
         <is>
           <t>Título livre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Bloqueante</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Subelemento de seção</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>section.code.coding.code</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Três códigos de seção do br-core-sumarioalta não estão no ValueSet doc-section-codes (required): 42347-5, 8654-6 e 54522-8.</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Levar ao BR-Core: códigos do doc-section-codes (candidatos 46241-6, 10183-2, 47420-5) ou binding extensible. Decisão pendente.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: D-39 resolvido no branch do BR-Core (section.code example, códigos do IPS)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UVSEtwhqSH6xEBzE8dBMwP
</commit_message>
<xml_diff>
--- a/comparativo/comparativo_sumarioalta_rnds_brcore.xlsx
+++ b/comparativo/comparativo_sumarioalta_rnds_brcore.xlsx
@@ -5736,7 +5736,7 @@
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>required: doc-section-codes; patternCodeableConcept = {"coding": [{"code": "42347-5", "system": "http://loinc.org"}]}</t>
+          <t>example: doc-section-codes; patternCodeableConcept = {"coding": [{"code": "42347-5", "system": "http://loinc.org"}]}</t>
         </is>
       </c>
       <c r="M15" s="6" t="inlineStr">
@@ -6668,7 +6668,7 @@
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>required: doc-section-codes; patternCodeableConcept = {"coding": [{"code": "57852-6", "system": "http://loinc.org"}]}</t>
+          <t>example: doc-section-codes; patternCodeableConcept = {"coding": [{"code": "57852-6", "system": "http://loinc.org"}]}</t>
         </is>
       </c>
       <c r="M28" s="6" t="inlineStr">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="L41" s="5" t="inlineStr">
         <is>
-          <t>required: doc-section-codes; patternCodeableConcept = {"coding": [{"code": "48765-2", "system": "http://loinc.org"}]}</t>
+          <t>example: doc-section-codes; patternCodeableConcept = {"coding": [{"code": "48765-2", "system": "http://loinc.org"}]}</t>
         </is>
       </c>
       <c r="M41" s="6" t="inlineStr">
@@ -8524,7 +8524,7 @@
       </c>
       <c r="L54" s="5" t="inlineStr">
         <is>
-          <t>required: doc-section-codes; patternCodeableConcept = {"coding": [{"code": "47519-4", "system": "http://loinc.org"}]}</t>
+          <t>example: doc-section-codes; patternCodeableConcept = {"coding": [{"code": "47519-4", "system": "http://loinc.org"}]}</t>
         </is>
       </c>
       <c r="M54" s="6" t="inlineStr">
@@ -9452,7 +9452,7 @@
       </c>
       <c r="L67" s="5" t="inlineStr">
         <is>
-          <t>required: doc-section-codes; patternCodeableConcept = {"coding": [{"code": "8654-6", "system": "http://loinc.org"}]}</t>
+          <t>example: doc-section-codes; patternCodeableConcept = {"coding": [{"code": "8654-6", "system": "http://loinc.org"}]}</t>
         </is>
       </c>
       <c r="M67" s="6" t="inlineStr">
@@ -10380,7 +10380,7 @@
       </c>
       <c r="L80" s="5" t="inlineStr">
         <is>
-          <t>required: doc-section-codes; patternCodeableConcept = {"coding": [{"code": "18776-5", "system": "http://loinc.org"}]}</t>
+          <t>example: doc-section-codes; patternCodeableConcept = {"coding": [{"code": "18776-5", "system": "http://loinc.org"}]}</t>
         </is>
       </c>
       <c r="M80" s="6" t="inlineStr">
@@ -11308,7 +11308,7 @@
       </c>
       <c r="L93" s="5" t="inlineStr">
         <is>
-          <t>required: doc-section-codes; patternCodeableConcept = {"coding": [{"code": "54522-8", "system": "http://loinc.org"}]}</t>
+          <t>example: doc-section-codes; patternCodeableConcept = {"coding": [{"code": "47420-5", "system": "http://loinc.org"}]}</t>
         </is>
       </c>
       <c r="M93" s="6" t="inlineStr">
@@ -14403,12 +14403,12 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Três códigos de seção do br-core-sumarioalta não estão no ValueSet doc-section-codes (required): 42347-5, 8654-6 e 54522-8.</t>
+          <t>br-core-composition liga section.code ao ValueSet doc-section-codes como required (no R4 e no IPS é example); 42347-5, 8654-6 e 54522-8 não estão no ValueSet.</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Levar ao BR-Core: códigos do doc-section-codes (candidatos 46241-6, 10183-2, 47420-5) ou binding extensible. Decisão pendente.</t>
+          <t>Corrigido no branch: binding example, como no IPS; capacidadeFuncional com o código do IPS 47420-5.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: perfis RNDS de restrição, CapabilityStatement e página para implementadores
- rnds-sumarioalta (parent br-core-sumarioalta, impõe clinical-document-composition),
  rnds-internacao (parent br-core-encounter), rnds-documento-sumarioalta
  (parent clinical-document-bundle): só cardinalidades, valores fixos e invariantes
- CapabilityStatement rnds-servidor-sumarioalta
- Página Implementação na RNDS; índice, estrutura, recomendações e README atualizados
- Exemplos com os perfis RNDS e raça/cor no paciente (D-40)
- Correções do BR-Core referidas ao main (9cf1bc9), não mais à branch
- json/: exemplos, perfis RNDS e pacotes atualizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UVSEtwhqSH6xEBzE8dBMwP
</commit_message>
<xml_diff>
--- a/comparativo/comparativo_sumarioalta_rnds_brcore.xlsx
+++ b/comparativo/comparativo_sumarioalta_rnds_brcore.xlsx
@@ -635,7 +635,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>BR-Core corrigido: branch fix/sumarioalta-capacidadefuncional do repositório br.org.hl7.fhir.core (snapshot gerado pelo SUSHI 3.20.1), ainda não publicado.</t>
+          <t>BR-Core corrigido: main do BR-Core (9cf1bc9) do repositório br.org.hl7.fhir.core (snapshot gerado pelo SUSHI 3.20.1), ainda não publicado.</t>
         </is>
       </c>
     </row>
@@ -782,7 +782,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>SA-IG em snapshot × pacote BR-Core 1.3.0 em snapshot × R4 × BR-Core corrigido (branch).</t>
+          <t>SA-IG em snapshot × pacote BR-Core 1.3.0 em snapshot × R4 × BR-Core corrigido (main).</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Discriminador profile em code e system https://loinc.org/: nenhuma instância valida (D-01, D-02). Corrigido no branch.</t>
+          <t>Discriminador profile em code e system https://loinc.org/: nenhuma instância valida (D-01, D-02). Corrigido no main do BR-Core.</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Correção no branch do BR-Core.</t>
+          <t>Correção no main do BR-Core do BR-Core.</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1175,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>br-core-bundle-documento criado no branch; segue o clinical-document-bundle.</t>
+          <t>br-core-bundle-documento criado no main do BR-Core; segue o clinical-document-bundle.</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
-          <t>BR-Core corrigido (branch) card.</t>
+          <t>BR-Core corrigido (main) card.</t>
         </is>
       </c>
       <c r="L1" s="4" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="P16" s="5" t="inlineStr">
         <is>
-          <t>Correção no branch fix/sumarioalta-capacidadefuncional do BR-Core: discriminador pattern em code.</t>
+          <t>Corrigido no main do BR-Core (9cf1bc9): discriminador pattern em code.</t>
         </is>
       </c>
       <c r="Q16" s="5" t="inlineStr">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
-          <t>BR-Core corrigido (branch) card.</t>
+          <t>BR-Core corrigido (main) card.</t>
         </is>
       </c>
       <c r="L1" s="4" t="inlineStr">
@@ -5832,7 +5832,7 @@
       </c>
       <c r="P16" s="5" t="inlineStr">
         <is>
-          <t>Corrigido no branch: http://loinc.org.</t>
+          <t>Corrigido no main do BR-Core: http://loinc.org.</t>
         </is>
       </c>
       <c r="Q16" s="5" t="inlineStr">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Corrigido no branch: http://loinc.org.</t>
+          <t>Corrigido no main do BR-Core: http://loinc.org.</t>
         </is>
       </c>
       <c r="Q29" s="5" t="inlineStr">
@@ -7692,7 +7692,7 @@
       </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Corrigido no branch: http://loinc.org.</t>
+          <t>Corrigido no main do BR-Core: http://loinc.org.</t>
         </is>
       </c>
       <c r="Q42" s="5" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="P55" s="5" t="inlineStr">
         <is>
-          <t>Corrigido no branch: http://loinc.org.</t>
+          <t>Corrigido no main do BR-Core: http://loinc.org.</t>
         </is>
       </c>
       <c r="Q55" s="5" t="inlineStr">
@@ -9548,7 +9548,7 @@
       </c>
       <c r="P68" s="5" t="inlineStr">
         <is>
-          <t>Corrigido no branch: http://loinc.org.</t>
+          <t>Corrigido no main do BR-Core: http://loinc.org.</t>
         </is>
       </c>
       <c r="Q68" s="5" t="inlineStr">
@@ -10476,7 +10476,7 @@
       </c>
       <c r="P81" s="5" t="inlineStr">
         <is>
-          <t>Corrigido no branch: http://loinc.org.</t>
+          <t>Corrigido no main do BR-Core: http://loinc.org.</t>
         </is>
       </c>
       <c r="Q81" s="5" t="inlineStr">
@@ -11172,7 +11172,7 @@
       </c>
       <c r="P91" s="5" t="inlineStr">
         <is>
-          <t>br-core-capacidadefuncional (correção no branch).</t>
+          <t>br-core-capacidadefuncional (correção no main do BR-Core).</t>
         </is>
       </c>
       <c r="Q91" s="5" t="inlineStr">
@@ -11404,7 +11404,7 @@
       </c>
       <c r="P94" s="5" t="inlineStr">
         <is>
-          <t>Corrigido no branch: http://loinc.org.</t>
+          <t>Corrigido no main do BR-Core: http://loinc.org.</t>
         </is>
       </c>
       <c r="Q94" s="5" t="inlineStr">
@@ -13598,7 +13598,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Correção no branch fix/sumarioalta-capacidadefuncional do BR-Core: discriminador pattern em code.</t>
+          <t>Corrigido no main do BR-Core (9cf1bc9): discriminador pattern em code.</t>
         </is>
       </c>
     </row>
@@ -13652,7 +13652,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Corrigido no branch: http://loinc.org.</t>
+          <t>Corrigido no main do BR-Core: http://loinc.org.</t>
         </is>
       </c>
     </row>
@@ -13922,7 +13922,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>br-core-capacidadefuncional (correção no branch).</t>
+          <t>br-core-capacidadefuncional (correção no main do BR-Core).</t>
         </is>
       </c>
     </row>
@@ -14408,7 +14408,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Corrigido no branch: binding example, como no IPS; capacidadeFuncional com o código do IPS 47420-5.</t>
+          <t>Corrigido no main do BR-Core: binding example, como no IPS; capacidadeFuncional com o código do IPS 47420-5.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scripts: fontes do mapa da estrutura alinhadas à página (numeração AC/DT na planilha; frase dos débitos no gerador)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UVSEtwhqSH6xEBzE8dBMwP
</commit_message>
<xml_diff>
--- a/comparativo/comparativo_sumarioalta_rnds_brcore.xlsx
+++ b/comparativo/comparativo_sumarioalta_rnds_brcore.xlsx
@@ -967,7 +967,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Discriminador profile em code e system https://loinc.org/: nenhuma instância valida (D-01, D-02). Corrigido no main do BR-Core.</t>
+          <t>Discriminador profile em code e system https://loinc.org/: nenhuma instância valida (AC-01, AC-02). Corrigido no main do BR-Core.</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Concorda e acrescenta que o br-core-patient exige CPF (1..1), o que impede o CNS provisório (D-03).</t>
+          <t>Concorda e acrescenta que o br-core-patient exige CPF (1..1), o que impede o CNS provisório (AC-03).</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">

</xml_diff>